<commit_message>
Update UI & animation for webapp, redesign landing page
</commit_message>
<xml_diff>
--- a/public/mau_cau_hoi.xlsx
+++ b/public/mau_cau_hoi.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Danh_Sach_Cau_Hoi" sheetId="1" r:id="rId1"/>
+    <sheet name="Questions" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A96"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,32 +406,482 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Đồng chí cảm thấy môi trường học tập và sinh hoạt hiện tại thế nào?</v>
+        <v>Đồng chí đánh giá mức độ khó của các nội dung huấn luyện trong tuần qua như thế nào?</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Đồng chí có mức độ hài lòng ra sao với chất lượng bữa ăn hàng ngày?</v>
+        <v>Đồng chí có gặp khó khăn gì trong việc thực hiện chế độ nền nếp chính quy tại đơn vị không?</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Đồng chí có gặp khó khăn gì trong công tác huấn luyện tại đơn vị không?</v>
+        <v>Đồng chí cảm thấy thế nào về cường độ huấn luyện hiện tại của đơn vị?</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Hoàn cảnh gia đình của đồng chí hiện tại có ổn định không? Có điều gì khiến đồng chí phải băn khoăn không?</v>
+        <v>Đồng chí có ý kiến gì về phương pháp giảng dạy của các cán bộ huấn luyện không?</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Mối quan hệ giữa đồng chí với đồng đội và chỉ huy các cấp đang như thế nào?</v>
+        <v>Đồng chí có cảm thấy mình đang tiến bộ hơn sau mỗi buổi tập không?</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Kỷ luật quân đội có gây áp lực quá lớn đối với đồng chí không?</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Đồng chí có nắm chắc các nội dung an toàn trong huấn luyện không?</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Đồng chí có đề xuất gì để nâng cao chất lượng huấn luyện tại trung đội không?</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Đồng chí có cảm thấy hăng hái khi tham gia các buổi tập hành quân không?</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Việc chấp hành giờ giấc nội vụ có gây khó khăn gì cho đồng chí không?</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Đồng chí có hài lòng với chất lượng bữa ăn tại bếp ăn tập thể không?</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Chế độ nghỉ ngơi, sinh hoạt của đồng chí có được đảm bảo đúng quy định không?</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Đồng chí có gặp vấn đề gì về sức khỏe trong thời gian gần đây không?</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Môi trường sinh hoạt tại đơn vị có đảm bảo vệ sinh và thông thoáng không?</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Đồng chí có thường xuyên tham gia các hoạt động thể dục thể thao không?</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Việc cấp phát nhu yếu phẩm tại đơn vị có đầy đủ và kịp thời không?</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Đồng chí có cảm thấy ngủ đủ giấc trong môi trường quân ngũ không?</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Đồng chí có gặp khó khăn gì trong việc thích nghi với khí hậu tại nơi đóng quân không?</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Hoạt động tăng gia sản xuất có giúp đồng chí giải tỏa căng thẳng không?</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Đồng chí có nhận được sự quan tâm đúng mức từ quân y đơn vị khi ốm đau không?</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Hoàn cảnh gia đình hiện tại có điều gì khiến đồng chí phải lo lắng không?</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Đồng chí có thường xuyên liên lạc về nhà để thăm hỏi gia đình không?</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Đồng chí có nhận được sự ủng hộ từ gia đình khi tham gia nghĩa vụ quân sự không?</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Đồng chí có cảm thấy nhớ nhà quá mức ảnh hưởng đến công tác không?</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Trước khi nhập ngũ, đồng chí có gặp vướng mắc gì về tình cảm cá nhân chưa giải quyết không?</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Đồng chí có dự định gì cho gia đình sau khi hoàn thành nghĩa vụ quân sự không?</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Gia đình đồng chí có đang gặp khó khăn về kinh tế hay chính sách gì không?</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Đồng chí có cảm thấy yên tâm công tác khi biết gia đình ở quê nhà ổn định không?</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Đồng chí có nhận được thư từ hay quà gửi từ người thân thường xuyên không?</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Đồng chí có cảm thấy áp lực từ những mong đợi của gia đình đối với mình không?</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Mối quan hệ của đồng chí với các chiến sĩ cùng tiểu đội như thế nào?</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Đồng chí có nhận được sự giúp đỡ từ đồng đội khi gặp khó khăn không?</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Trong đơn vị có hiện tượng mất đoàn kết hay chia rẽ nội bộ không?</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Đồng chí có tin tưởng vào sự chỉ huy và dẫn dắt của tiểu đội trưởng không?</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Đồng chí cảm thấy cán bộ trung đội có gần gũi và sâu sát với chiến sĩ không?</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Khi có mâu thuẫn với đồng đội, đồng chí thường giải quyết theo cách nào?</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Đồng chí có cảm thấy mình là một phần quan trọng của tập thể đơn vị không?</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Đồng chí có sẵn sàng giúp đỡ đồng đội khác trong học tập và công tác không?</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Có bao giờ đồng chí cảm thấy bị cô lập trong môi trường đơn vị không?</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Đồng chí đánh giá thế nào về tinh thần tương thân tương ái tại đơn vị mình?</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Đồng chí có hiểu rõ mục đích và ý nghĩa của việc thực hiện nghĩa vụ quân sự không?</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Đồng chí có cảm thấy tự hào khi được đứng trong hàng ngũ Quân đội nhân dân Việt Nam không?</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Động lực lớn nhất giúp đồng chí vượt qua những ngày huấn luyện gian khổ là gì?</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Đồng chí có mục tiêu phấn đấu để trở thành Đảng viên trong thời gian tại ngũ không?</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Đồng chí có ý định thi vào các trường quân đội hoặc phục vụ lâu dài không?</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Đồng chí có cảm thấy những kiến thức quân sự đang học có ích cho tương lai không?</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Đồng chí có tinh thần sẵn sàng nhận và hoàn thành mọi nhiệm vụ được giao không?</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Đồng chí có tin tưởng vào vũ khí và trang bị kỹ thuật được cấp phát không?</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Đồng chí có cảm nhận được sự thay đổi tích cực của bản thân từ khi nhập ngũ không?</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Nếu được chọn lại, đồng chí vẫn sẽ hăng hái lên đường nhập ngũ chứ?</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Đồng chí có yêu thích các buổi sinh hoạt văn nghệ, đọc báo tại đơn vị không?</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Các chương trình phát thanh nội bộ có cung cấp thông tin hữu ích cho đồng chí không?</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Đồng chí có thường xuyên sử dụng phòng đọc sách hay thư viện của đơn vị không?</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Các trò chơi quân sự và hoạt động tập thể có giúp đồng chí gắn kết hơn không?</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Đồng chí có cảm thấy các buổi sinh hoạt ngày chính trị văn hóa tinh thần có hiệu quả không?</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Đồng chí có điều gì muốn đề đạt trực tiếp với chỉ huy cấp trên không?</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Đồng chí có cảm thấy công tâm trong việc bình xét thi đua khen thưởng không?</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Có vấn đề gì trong đơn vị mà đồng chí thấy cần phải thay đổi ngay không?</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Đồng chí có lo lắng về việc tìm kiếm việc làm sau khi xuất ngũ không?</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Đồng chí có cảm thấy mình được tôn trọng khi ở trong môi trường quân ngũ không?</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Đồng chí có nhận xét gì về việc sử dụng thời gian rảnh rỗi tại đơn vị?</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Đồng chí có cảm thấy an tâm khi thực hiện các nhiệm vụ canh gác, tuần tra không?</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Có lúc nào đồng chí cảm thấy chán nản và muốn bỏ cuộc không?</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Đồng chí mong muốn đơn vị tổ chức thêm những hoạt động ngoại khóa nào?</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Đồng chí có cảm thấy hệ thống khảo sát này là cơ hội tốt để bày tỏ tâm tư không?</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Đồng chí có nhận thấy sự gương mẫu của các cán bộ đảng viên trong đơn vị không?</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Việc quản lý vũ khí trang bị tại đơn vị có nghiêm túc và an toàn không?</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Đồng chí có nắm vững 12 điều kỷ luật khi quan hệ với nhân dân không?</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Đồng chí có tham gia đầy đủ các buổi học chính trị trong tháng không?</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Đồng chí đánh giá thế nào về công tác vệ sinh môi trường quanh doanh trại?</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Đồng chí có cảm thấy tự tin khi thực hiện bài bắn đạn thật không?</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Mối quan hệ giữa đơn vị và nhân dân nơi đóng quân có tốt không?</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Đồng chí có ý kiến gì về việc quản lý sử dụng điện thoại tại đơn vị?</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Đồng chí có nhận thấy sự quan tâm của cấp trên đến đời sống chiến sĩ không?</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Đồng chí có thường xuyên theo dõi tin tức thời sự trên truyền hình quân đội không?</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Đồng chí có cảm thấy các bài học về truyền thống đơn vị có ý nghĩa không?</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Việc bảo quản vũ khí (lau chùi súng) có thực hiện đúng quy định hàng ngày không?</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Đồng chí có sẵn sàng tham gia các nhiệm vụ phòng chống thiên tai, cứu hộ không?</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Đồng chí có cảm thấy an toàn khi tham gia các bài tập ném lựu đạn thật không?</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Đồng chí có nắm vững các chức trách, nhiệm vụ của mình khi trực ban không?</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Việc chi trả phụ cấp hàng tháng có đúng hạn và đầy đủ không?</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Đồng chí có cảm thấy hãnh diện khi mặc bộ quân phục trên người không?</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Đồng chí có nhận xét gì về văn hóa ứng xử của các cán bộ trẻ mới về đơn vị?</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Các hoạt động ngày nghỉ có phong phú và hấp dẫn đồng chí không?</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Đồng chí có cảm nhận được sự công bằng trong việc phân công nhiệm vụ lao động không?</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Đồng chí có muốn học thêm một nghề nào đó trong thời gian tại ngũ không?</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Đồng chí có tự tin về khả năng bơi lội của mình nếu tham gia huấn luyện dưới nước không?</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Việc cắt tóc, xưng hô chào hỏi có được thực hiện nghiêm túc trong đơn vị không?</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Đồng chí có nắm chắc các dấu hiệu nhận biết về diễn biến tâm lý tiêu cực ở đồng đội không?</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Đồng chí có thường xuyên tự học, tự rèn thêm ngoài giờ huấn luyện không?</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Đồng chí có cảm thấy môi trường quân đội giúp mình trưởng thành hơn không?</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Đồng chí có mong muốn được thăm gia đình trong những dịp lễ đặc biệt không?</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Đồng chí có hiểu rõ quyền lợi và nghĩa vụ của một người chiến sĩ không?</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Đồng chí có cảm nhận được sự ấm áp của tình đồng chí như trong một gia đình không?</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Đồng chí có quyết tâm đạt danh hiệu Chiến sĩ tiên tiến trong năm nay không?</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A96"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>